<commit_message>
New cad design added
</commit_message>
<xml_diff>
--- a/Hardware/BOM/STM32+ESP32BOM (2)_connector.xlsx
+++ b/Hardware/BOM/STM32+ESP32BOM (2)_connector.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Elconics\Projects\2025\stm32_learning_baord_v1\stm32_lb1_modified\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Elconics\Projects\2026\STM32_LB1\Elconics-Duino\Hardware\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0EF4A1BE-EA06-46C7-84C9-B1E3BDDFE9D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{552D7CDF-7053-4733-8385-EA29847A6303}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{51A68588-214E-4FF5-9276-A10186426552}"/>
+    <workbookView xWindow="1515" yWindow="1515" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{51A68588-214E-4FF5-9276-A10186426552}"/>
   </bookViews>
   <sheets>
     <sheet name="robu" sheetId="1" r:id="rId1"/>
@@ -1171,17 +1171,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31C964F8-F0E6-4962-8340-D41E7BAF16AF}">
   <dimension ref="A1:H34"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.88671875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="33.77734375" style="3" customWidth="1"/>
-    <col min="4" max="4" width="26.88671875" style="3" customWidth="1"/>
+    <col min="1" max="1" width="15.85546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="33.7109375" style="3" customWidth="1"/>
+    <col min="4" max="4" width="26.85546875" style="3" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="25.88671875" customWidth="1"/>
-    <col min="8" max="8" width="14.109375" customWidth="1"/>
+    <col min="7" max="7" width="25.85546875" customWidth="1"/>
+    <col min="8" max="8" width="14.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1207,7 +1207,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>107047</v>
       </c>
@@ -1233,7 +1233,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
@@ -1259,7 +1259,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>1415726</v>
       </c>
@@ -1285,7 +1285,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>1090076</v>
       </c>
@@ -1311,7 +1311,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>29</v>
       </c>
@@ -1337,7 +1337,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>34</v>
       </c>
@@ -1363,7 +1363,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>596592</v>
       </c>
@@ -1389,7 +1389,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>43</v>
       </c>
@@ -1415,7 +1415,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>48</v>
       </c>
@@ -1441,7 +1441,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>827881</v>
       </c>
@@ -1467,7 +1467,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>58</v>
       </c>
@@ -1493,7 +1493,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>63</v>
       </c>
@@ -1519,7 +1519,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>1859282</v>
       </c>
@@ -1545,7 +1545,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>78</v>
       </c>
@@ -1571,7 +1571,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>598591</v>
       </c>
@@ -1597,7 +1597,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>135</v>
       </c>
@@ -1623,7 +1623,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>141</v>
       </c>
@@ -1649,7 +1649,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>145</v>
       </c>
@@ -1675,7 +1675,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>150</v>
       </c>
@@ -1701,7 +1701,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>155</v>
       </c>
@@ -1727,7 +1727,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>158</v>
       </c>
@@ -1753,7 +1753,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>163</v>
       </c>
@@ -1779,7 +1779,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>1555127</v>
       </c>
@@ -1805,7 +1805,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>177</v>
       </c>
@@ -1831,7 +1831,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>182</v>
       </c>
@@ -1857,7 +1857,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>162032</v>
       </c>
@@ -1883,7 +1883,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>191</v>
       </c>
@@ -1909,7 +1909,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>197</v>
       </c>
@@ -1935,7 +1935,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>208</v>
       </c>
@@ -1961,7 +1961,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>1142274</v>
       </c>
@@ -1987,7 +1987,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>601600</v>
       </c>
@@ -2013,7 +2013,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>223</v>
       </c>
@@ -2039,7 +2039,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>228</v>
       </c>
@@ -2112,9 +2112,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A7DDE8D-819A-4D77-855B-F81BE43F235A}">
   <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2140,7 +2140,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>72</v>
       </c>
@@ -2166,7 +2166,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>85</v>
       </c>
@@ -2192,7 +2192,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>94</v>
       </c>
@@ -2218,7 +2218,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>111</v>
       </c>
@@ -2244,7 +2244,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>117</v>
       </c>
@@ -2270,7 +2270,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>167</v>
       </c>
@@ -2296,7 +2296,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>202</v>
       </c>
@@ -2339,9 +2339,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E43B6A3-60F7-4E67-9D8F-71D86F6D5327}">
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="24.28515625" customWidth="1"/>
+    <col min="2" max="2" width="36.28515625" customWidth="1"/>
+    <col min="3" max="3" width="23.5703125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -2367,7 +2372,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>4</v>
       </c>
@@ -2381,7 +2386,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>3</v>
       </c>
@@ -2395,7 +2400,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -2409,7 +2414,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -2423,7 +2428,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1</v>
       </c>
@@ -2437,7 +2442,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2</v>
       </c>
@@ -2451,7 +2456,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2</v>
       </c>
@@ -2465,7 +2470,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1</v>
       </c>
@@ -2479,7 +2484,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>1</v>
       </c>
@@ -2493,7 +2498,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B11" s="3"/>
     </row>
   </sheetData>

</xml_diff>